<commit_message>
Looping through inputs and searching for each one
</commit_message>
<xml_diff>
--- a/main/Locations.xlsx
+++ b/main/Locations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\unibuc mafia\UIPath\rpa-vacation-finder\main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDAD27E-512B-4D7A-B041-3031329AAADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C868443-FC33-42C0-8454-64F9D35E7C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{428E27FE-7ACA-403B-B9C4-319042B80A9C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ID</t>
   </si>
@@ -51,6 +51,12 @@
   </si>
   <si>
     <t>Tokyo</t>
+  </si>
+  <si>
+    <t>CheckInDate</t>
+  </si>
+  <si>
+    <t>CheckOutDate</t>
   </si>
 </sst>
 </file>
@@ -86,8 +92,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -422,16 +429,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75D5ADBC-BDEB-4D8E-8D02-D27D4BC087D6}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="39.85546875" customWidth="1"/>
     <col min="4" max="4" width="31.7109375" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,8 +449,14 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -452,8 +466,14 @@
       <c r="C2">
         <v>2</v>
       </c>
+      <c r="D2" s="1">
+        <v>46188</v>
+      </c>
+      <c r="E2" s="1">
+        <v>46195</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -462,6 +482,12 @@
       </c>
       <c r="C3">
         <v>6</v>
+      </c>
+      <c r="D3" s="1">
+        <v>46193</v>
+      </c>
+      <c r="E3" s="1">
+        <v>46280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added no rating fallback
</commit_message>
<xml_diff>
--- a/main/Locations.xlsx
+++ b/main/Locations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\unibuc mafia\UIPath\rpa-vacation-finder\main\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\curec\Documents\GitHub\rpa-vacation-finder\main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C868443-FC33-42C0-8454-64F9D35E7C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1667CA-120B-4056-91A6-6D19D473993C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{428E27FE-7ACA-403B-B9C4-319042B80A9C}"/>
+    <workbookView xWindow="870" yWindow="3210" windowWidth="21600" windowHeight="11295" xr2:uid="{428E27FE-7ACA-403B-B9C4-319042B80A9C}"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>ID</t>
   </si>
@@ -57,6 +57,15 @@
   </si>
   <si>
     <t>CheckOutDate</t>
+  </si>
+  <si>
+    <t>Brasov</t>
+  </si>
+  <si>
+    <t>Milano</t>
+  </si>
+  <si>
+    <t>Seoul</t>
   </si>
 </sst>
 </file>
@@ -429,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75D5ADBC-BDEB-4D8E-8D02-D27D4BC087D6}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -490,6 +499,57 @@
         <v>46280</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1">
+        <v>46065</v>
+      </c>
+      <c r="E4" s="1">
+        <v>46067</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <v>46126</v>
+      </c>
+      <c r="E5" s="1">
+        <v>46127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1">
+        <v>46210</v>
+      </c>
+      <c r="E6" s="1">
+        <v>46251</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Started working on exceptions
</commit_message>
<xml_diff>
--- a/main/Locations.xlsx
+++ b/main/Locations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\curec\Documents\GitHub\rpa-vacation-finder\main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1667CA-120B-4056-91A6-6D19D473993C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929FD85C-A0D3-415F-A4AE-5C89E6AE9558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="870" yWindow="3210" windowWidth="21600" windowHeight="11295" xr2:uid="{428E27FE-7ACA-403B-B9C4-319042B80A9C}"/>
+    <workbookView xWindow="3270" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{428E27FE-7ACA-403B-B9C4-319042B80A9C}"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>ID</t>
   </si>
@@ -47,25 +47,10 @@
     <t>NumberOfGuests</t>
   </si>
   <si>
-    <t>Barcelona</t>
-  </si>
-  <si>
-    <t>Tokyo</t>
-  </si>
-  <si>
     <t>CheckInDate</t>
   </si>
   <si>
     <t>CheckOutDate</t>
-  </si>
-  <si>
-    <t>Brasov</t>
-  </si>
-  <si>
-    <t>Milano</t>
-  </si>
-  <si>
-    <t>Seoul</t>
   </si>
 </sst>
 </file>
@@ -459,96 +444,31 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1">
-        <v>46188</v>
-      </c>
-      <c r="E2" s="1">
-        <v>46195</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1">
-        <v>46193</v>
-      </c>
-      <c r="E3" s="1">
-        <v>46280</v>
-      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-      <c r="D4" s="1">
-        <v>46065</v>
-      </c>
-      <c r="E4" s="1">
-        <v>46067</v>
-      </c>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1">
-        <v>46126</v>
-      </c>
-      <c r="E5" s="1">
-        <v>46127</v>
-      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6">
-        <v>4</v>
-      </c>
-      <c r="D6" s="1">
-        <v>46210</v>
-      </c>
-      <c r="E6" s="1">
-        <v>46251</v>
-      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>